<commit_message>
Update all report cards with corrected SS2 scores
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Balogun_Khadijat.xlsx
+++ b/report_cards/Report_Card_Balogun_Khadijat.xlsx
@@ -1515,11 +1515,11 @@
         <v>16</v>
       </c>
       <c r="H28" s="42" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I28" s="36" t="n"/>
       <c r="J28" s="42" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K28" s="36" t="n"/>
       <c r="L28" s="18">
@@ -1573,14 +1573,14 @@
       <c r="E29" s="35" t="n"/>
       <c r="F29" s="36" t="n"/>
       <c r="G29" s="42" t="n">
+        <v>14</v>
+      </c>
+      <c r="H29" s="42" t="n">
         <v>13</v>
-      </c>
-      <c r="H29" s="42" t="n">
-        <v>14</v>
       </c>
       <c r="I29" s="36" t="n"/>
       <c r="J29" s="42" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K29" s="36" t="n"/>
       <c r="L29" s="18">
@@ -1634,14 +1634,14 @@
       <c r="E30" s="35" t="n"/>
       <c r="F30" s="36" t="n"/>
       <c r="G30" s="42" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H30" s="42" t="n">
         <v>19</v>
       </c>
       <c r="I30" s="36" t="n"/>
       <c r="J30" s="42" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K30" s="36" t="n"/>
       <c r="L30" s="18">
@@ -2016,7 +2016,7 @@
         </is>
       </c>
       <c r="X38" s="43" t="n">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="Y38" s="30" t="n"/>
       <c r="Z38" s="30" t="n"/>
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="X39" s="43" t="n">
-        <v>79.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="Y39" s="30" t="n"/>
       <c r="Z39" s="30" t="n"/>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="X40" s="43" t="inlineStr">
         <is>
-          <t>79.56%</t>
+          <t>79.78%</t>
         </is>
       </c>
       <c r="Y40" s="30" t="n"/>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="I42" s="36" t="n"/>
       <c r="J42" s="42" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="K42" s="36" t="n"/>
       <c r="L42" s="18">
@@ -2220,11 +2220,11 @@
         <v>15</v>
       </c>
       <c r="H43" s="42" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I43" s="36" t="n"/>
       <c r="J43" s="42" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K43" s="36" t="n"/>
       <c r="L43" s="18">
@@ -2341,14 +2341,14 @@
       <c r="E46" s="35" t="n"/>
       <c r="F46" s="36" t="n"/>
       <c r="G46" s="42" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H46" s="42" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I46" s="36" t="n"/>
       <c r="J46" s="42" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="K46" s="36" t="n"/>
       <c r="L46" s="18">
@@ -2434,7 +2434,7 @@
       <c r="E48" s="35" t="n"/>
       <c r="F48" s="36" t="n"/>
       <c r="G48" s="44" t="n">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="H48" s="35" t="n"/>
       <c r="I48" s="35" t="n"/>
@@ -2466,7 +2466,7 @@
       <c r="E49" s="35" t="n"/>
       <c r="F49" s="36" t="n"/>
       <c r="G49" s="44" t="n">
-        <v>79.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="H49" s="35" t="n"/>
       <c r="I49" s="35" t="n"/>
@@ -2499,7 +2499,7 @@
       <c r="F50" s="36" t="n"/>
       <c r="G50" s="44" t="inlineStr">
         <is>
-          <t>79.56%</t>
+          <t>79.78%</t>
         </is>
       </c>
       <c r="H50" s="35" t="n"/>

</xml_diff>

<commit_message>
Fix Balogun: CSV base 569, Computer 65, Yoruba 84 = 718 (3rd)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Balogun_Khadijat.xlsx
+++ b/report_cards/Report_Card_Balogun_Khadijat.xlsx
@@ -1519,7 +1519,7 @@
       </c>
       <c r="I28" s="36" t="n"/>
       <c r="J28" s="42" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K28" s="36" t="n"/>
       <c r="L28" s="18">
@@ -1573,14 +1573,14 @@
       <c r="E29" s="35" t="n"/>
       <c r="F29" s="36" t="n"/>
       <c r="G29" s="42" t="n">
+        <v>13</v>
+      </c>
+      <c r="H29" s="42" t="n">
         <v>14</v>
-      </c>
-      <c r="H29" s="42" t="n">
-        <v>13</v>
       </c>
       <c r="I29" s="36" t="n"/>
       <c r="J29" s="42" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K29" s="36" t="n"/>
       <c r="L29" s="18">
@@ -1634,14 +1634,14 @@
       <c r="E30" s="35" t="n"/>
       <c r="F30" s="36" t="n"/>
       <c r="G30" s="42" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H30" s="42" t="n">
         <v>19</v>
       </c>
       <c r="I30" s="36" t="n"/>
       <c r="J30" s="42" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K30" s="36" t="n"/>
       <c r="L30" s="18">
@@ -2038,7 +2038,7 @@
         <v>17</v>
       </c>
       <c r="H39" s="42" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I39" s="36" t="n"/>
       <c r="J39" s="42" t="n">
@@ -2057,7 +2057,7 @@
       <c r="O39" s="36" t="n"/>
       <c r="P39" s="42" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>3rd</t>
         </is>
       </c>
       <c r="Q39" s="35" t="n"/>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="I42" s="36" t="n"/>
       <c r="J42" s="42" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K42" s="36" t="n"/>
       <c r="L42" s="18">
@@ -2220,11 +2220,11 @@
         <v>15</v>
       </c>
       <c r="H43" s="42" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I43" s="36" t="n"/>
       <c r="J43" s="42" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K43" s="36" t="n"/>
       <c r="L43" s="18">
@@ -2341,14 +2341,14 @@
       <c r="E46" s="35" t="n"/>
       <c r="F46" s="36" t="n"/>
       <c r="G46" s="42" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H46" s="42" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I46" s="36" t="n"/>
       <c r="J46" s="42" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="K46" s="36" t="n"/>
       <c r="L46" s="18">

</xml_diff>

<commit_message>
Fix Balogun Civic 96 (not 100), English 89, total 752 3rd
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Balogun_Khadijat.xlsx
+++ b/report_cards/Report_Card_Balogun_Khadijat.xlsx
@@ -1512,14 +1512,14 @@
       <c r="E28" s="35" t="n"/>
       <c r="F28" s="36" t="n"/>
       <c r="G28" s="42" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H28" s="42" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I28" s="36" t="n"/>
       <c r="J28" s="42" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K28" s="36" t="n"/>
       <c r="L28" s="18">
@@ -1634,14 +1634,14 @@
       <c r="E30" s="35" t="n"/>
       <c r="F30" s="36" t="n"/>
       <c r="G30" s="42" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H30" s="42" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I30" s="36" t="n"/>
       <c r="J30" s="42" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K30" s="36" t="n"/>
       <c r="L30" s="18">

</xml_diff>